<commit_message>
[Big Orange] - Added Alexa ShutdownIntent to initiate robot shutdown via voice command - Added ShutdownIntent handler and samples ("start shutting down", "initiate shutdown") to Alexa skill - Added skill.json for Alexa skill metadata - Configured AWS IoT endpoint and BigOrange certificate paths in Alexa lambda - Added moveTosFloat() and moveTosFloatWithYaw() to SlamtecDll for multi-waypoint navigation using RobotLocations struct - Added RobotLocation / RobotLocations structs (up to 10 waypoints) to SlamtecDll.h - Fixed recoverLocalization() to not block on waitUntilDone() - Added disparity_filtering.cpp for depth camera stereo disparity post-processing - Updated .gitignore and docs (presentation, battery discharge, langgraph diagram, persona pptx)
</commit_message>
<xml_diff>
--- a/doc/RobotBatteryDischarge.xlsx
+++ b/doc/RobotBatteryDischarge.xlsx
@@ -1,33 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/adda657fb66bcada/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\Users\Jim\Documents\git\big-orange\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C1A574B-218D-4F7A-9C31-C93EECDB41F7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E6F7412-3EAC-442E-AB77-E771466F366A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="15435" xr2:uid="{DF79FCFF-E377-4858-99E4-B5506EAA46F7}"/>
+    <workbookView xWindow="2325" yWindow="1575" windowWidth="26985" windowHeight="16770" xr2:uid="{DF79FCFF-E377-4858-99E4-B5506EAA46F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$A$4:$A$8</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$B$4:$B$8</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -143,6 +138,7 @@
               <a:rPr lang="en-US" baseline="0"/>
               <a:t> Orange Battery Discharge</a:t>
             </a:r>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -184,14 +180,9 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:v>Measured</c:v>
-          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
+              <a:noFill/>
               <a:round/>
             </a:ln>
             <a:effectLst/>
@@ -211,6 +202,51 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$A$4:$A$8</c:f>
@@ -218,19 +254,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>12</c:v>
+                  <c:v>11.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11.5</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10.4</c:v>
+                  <c:v>10.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.24</c:v>
+                  <c:v>9.1</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>7</c:v>
+                  <c:v>7.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -262,92 +298,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B19C-43A6-8BAF-FF471C084509}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Fitted Curve</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent2"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$C$11:$C$15</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>11.5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>10.4</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>9.24</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>7</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$D$11:$D$15</c:f>
-              <c:numCache>
-                <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>0.97868214408221998</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.79006348344203703</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.47564939889198793</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.25300875819801499</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.2597546885365712E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E7C3-48F3-A48B-D0AEB2A89AC6}"/>
+              <c16:uniqueId val="{00000000-466F-46EE-8498-2B0E6A43C725}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -359,11 +310,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="466122424"/>
-        <c:axId val="466127016"/>
+        <c:axId val="422931584"/>
+        <c:axId val="422934464"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="466122424"/>
+        <c:axId val="422931584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -420,12 +371,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="466127016"/>
+        <c:crossAx val="422934464"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="466127016"/>
+        <c:axId val="422934464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -482,7 +433,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="466122424"/>
+        <c:crossAx val="422931584"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -494,39 +445,15 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
     <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
@@ -1122,23 +1049,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>128587</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>309562</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>333375</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>14287</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>4762</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>185737</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B7CB7D1A-B2C9-4E04-8EE7-05C2F76EB74A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9AB69A3A-0E11-4B7A-F05C-55C4B8C7984A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1457,52 +1384,52 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE806310-0037-4405-AF5C-E623CBC8C53F}">
   <dimension ref="A4:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.703125" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>11.5</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1">
         <v>0.75</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="B6" s="1">
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>9.24</v>
+        <v>9.1</v>
       </c>
       <c r="B7" s="1">
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="B8" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1516,7 +1443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1524,14 +1451,14 @@
         <v>1</v>
       </c>
       <c r="C11">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="D11" s="2">
-        <f xml:space="preserve"> -0.1700162 - (-0.005948003/-0.3530656)*(1 - EXP(0.3530656*C11))</f>
-        <v>0.97868214408221998</v>
+        <f xml:space="preserve">  0.0349*C11^2 - 0.4255*C11 + 1.2308</f>
+        <v>0.99114400000000069</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
@@ -1539,14 +1466,14 @@
         <v>0.75</v>
       </c>
       <c r="C12">
-        <v>11.5</v>
+        <v>11</v>
       </c>
       <c r="D12" s="2">
-        <f t="shared" ref="D12:D15" si="0" xml:space="preserve"> -0.1700162 - (-0.005948003/-0.3530656)*(1 - EXP(0.3530656*C12))</f>
-        <v>0.79006348344203703</v>
+        <f t="shared" ref="D12:D15" si="0" xml:space="preserve">  0.0349*C12^2 - 0.4255*C12 + 1.2308</f>
+        <v>0.77319999999999967</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1554,14 +1481,14 @@
         <v>0.5</v>
       </c>
       <c r="C13">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="D13" s="2">
         <f t="shared" si="0"/>
-        <v>0.47564939889198793</v>
+        <v>0.49339900000000014</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1</v>
       </c>
@@ -1569,14 +1496,14 @@
         <v>0.25</v>
       </c>
       <c r="C14">
-        <v>9.24</v>
+        <v>9.1</v>
       </c>
       <c r="D14" s="2">
         <f t="shared" si="0"/>
-        <v>0.25300875819801499</v>
+        <v>0.24881899999999968</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>0</v>
       </c>
@@ -1584,11 +1511,11 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="D15" s="2">
         <f t="shared" si="0"/>
-        <v>1.2597546885365712E-2</v>
+        <v>2.6749999999997609E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>